<commit_message>
feat: kasboek-style Excel output, dual-account support, 2025 processing
- Rebuilt Excel output to match old kasboek: 4 colour-coded blocks
  (INKOMEN / VASTE LASTEN / DAGELIJKS / OVERIG) + SAMENVATTING + NETTO
- Added --year YYYY flag to filter to a single year
- Added Interne Overboeking detection for betaalrekening <-> spaarrekening
  transfers; these appear in Transacties but are excluded from all totals
- Replaced Jaar Overzicht with Jaar Samenvatting: totals + % van inkomen
- Output file named boekhouding_YYYY.xlsx when --year is used
- Richer terminal summary: inkomen | vaste lasten | dagelijks | netto per month
- Updated rules.xlsx to canonical category system (35 rules)
- Updated README and CLAUDE.md with current state and next-session checklist

2025 processing: 49% coverage on first run; rules gap-fill pending

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bookkeeping/rules.xlsx
+++ b/bookkeeping/rules.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Diversen</t>
+          <t>Online Winkelen</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Diversen</t>
+          <t>Online Winkelen</t>
         </is>
       </c>
     </row>
@@ -677,7 +677,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Verzekeringen</t>
+          <t>Zorgverzekering</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Sport &amp; Fitness</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Sport</t>
+          <t>Sport &amp; Fitness</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Telefoon</t>
+          <t>Telefoon &amp; Internet</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Vaste Lasten</t>
+          <t>Diversen</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Inkomen</t>
+          <t>Salaris</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Inkomen</t>
+          <t>Salaris</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Kamerhuur</t>
+          <t>Huur &amp; Wonen</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Eten &amp; Drinken</t>
+          <t>Tabak</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Eten &amp; Drinken</t>
+          <t>Tabak</t>
         </is>
       </c>
     </row>
@@ -857,7 +857,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Diversen</t>
+          <t>Cultuur &amp; Entertainment</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: 2025 rules gap-fill + onbekend rows + controle sheet + totaal kosten
- rules.xlsx: 7 stale categories migrated + 29 new keywords (74% coverage)
- CLAUDE.md: category list synced with 2026 restructure
- Maand Overzicht: ONBEKEND section (Onbekend Inkomen/Uitgaven rows)
- Maand Overzicht: Totaal Kosten rij (lichtroze, positief bedrag)
- Onbekend sheet: sorteer op abs(totaal) hoog-naar-laag + autofilter op databereik
- Nieuw: Controle sheet met per-maand reconciliatie (5e tab)
- BACKLOG: Now bijgewerkt naar huidige staat

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bookkeeping/rules.xlsx
+++ b/bookkeeping/rules.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -533,7 +533,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Online Winkelen</t>
+          <t>Dagelijks Overig</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Online Winkelen</t>
+          <t>Dagelijks Overig</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Huur &amp; Wonen</t>
+          <t>Huur</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Eten &amp; Drinken</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Tabak</t>
+          <t>Eten &amp; Drinken</t>
         </is>
       </c>
     </row>
@@ -870,6 +870,354 @@
       <c r="B36" t="inlineStr">
         <is>
           <t>Diversen</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>hoyng</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Huur</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>j.p.q. hoyng</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Huur</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>optimal solutions</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Salaris</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>d. van rhijn</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Familie &amp; Giften</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>dhr. c. van rhijn</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Familie &amp; Giften</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>christiaan van rhijn</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Familie &amp; Giften</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>rhijn d van</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Familie &amp; Giften</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>j. van rhijn</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Familie &amp; Giften</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>trefpunt</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>tkmbv</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Dagelijks Overig</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>biblioth</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Cultuur &amp; Entertainment</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>dizzy duck</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>kruidvat</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Gezondheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>decathlon</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Sport &amp; Fitness</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ka pompenburg</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>coffeeshop</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Dagelijks Overig</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>nyx sanitronics</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Bankkosten</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>donkeyr</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Dagelijks Overig</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>alepa</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>night2night</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Uitgaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>rente en/of kosten</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Bankkosten</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>grill n spice</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>leiden 4208</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>juni lekkernijen</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>eerste kamer</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>revolut</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Dagelijks Overig</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>istanbul doner</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>delirium</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Uitgaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>tabakspeciaalzaak</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: tkmbv -> Gezondheid, ka pompenburg -> Kapper
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bookkeeping/rules.xlsx
+++ b/bookkeeping/rules.xlsx
@@ -989,7 +989,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Dagelijks Overig</t>
+          <t>Gezondheid</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>OV &amp; Reizen</t>
+          <t>Kapper</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: 40 nieuwe regels vanuit Onbekend 2026 (94% coverage)
Toegevoegd: salaris, ov/reizen, WbW, gezondheid, abonnementen,
onderhoud, boodschappen, uitgaan, eten categorieën voor 2026 merchants.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bookkeeping/rules.xlsx
+++ b/bookkeeping/rules.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B65"/>
+  <dimension ref="A1:B105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1216,6 +1216,486 @@
         </is>
       </c>
       <c r="B65" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>optimal data</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Salaris</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>cjc vincenten</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>trip.com</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>ryanair</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>boho hostel</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>malta public</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>mark molenaar</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>WbW</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>deutman</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>WbW</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>dijkje</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>WbW</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>aab inz tikkie</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>WbW</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>o'neill</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>WbW</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>ccv*nfk</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>WbW</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>amazon eu</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>WbW</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>zoo bar</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>WbW</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>lautenschutz</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>WbW</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>tfl travel</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>WbW</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>linen and co</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>WbW</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>mm the corner</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Gezondheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>crave nest</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Gezondheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>gozo highspeed</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Gezondheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>renssen sigaren</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Gezondheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>salsashop</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Gezondheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>space bal</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Gezondheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>st johns co</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Gezondheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>sijf</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Gezondheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>shop delft</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Gezondheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>studenten corps</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Abonnementen</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>siebenhaar</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Dagelijks Overig</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Onderhoud</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>groen in</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Boodschappen</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>vader kleinjan</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Uitgaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>piccolo padre</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Uitgaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>marsamxetto</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Uitgaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>fort st elmo</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Uitgaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>halal food</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>grand master</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>princessa polaki</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>spar savoy</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>vessel 11</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>cdl chocolate</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
         <is>
           <t>Eten &amp; Drinken</t>
         </is>

</xml_diff>

<commit_message>
refactor: Onbekend + Diversen -> Dagelijks Overig
Alle niet-gematchte transacties vallen nu in Dagelijks Overig.
Diversen verwijderd als aparte categorie. Onbekend-sheet verwijderd.
Controle-sheet: kolommen Onbekend Inc/Uit verwijderd.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bookkeeping/rules.xlsx
+++ b/bookkeeping/rules.xlsx
@@ -773,7 +773,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Diversen</t>
+          <t>Dagelijks Overig</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Diversen</t>
+          <t>Dagelijks Overig</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: interne overboekingen, ZZP opname, beleggen toegevoegd
- ZZP Opname (INKOMEN): matcht op knabnl in beschrijving via config.json
- Beleggen (OVERIG): matcht op degiro/de giro; telt niet mee in Totaal Kosten
- Interne Overboeking: nu zichtbaar als grijze rij in Maand Overzicht
- config.json: IBAN-regels + auto-detect eigen rekeningnummers uit TAB-bestanden

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bookkeeping/rules.xlsx
+++ b/bookkeeping/rules.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B105"/>
+  <dimension ref="A1:B107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1698,6 +1698,30 @@
       <c r="B105" t="inlineStr">
         <is>
           <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>degiro</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Beleggen</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>de giro</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Beleggen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: categorisatieregels uitgebreid (106 → 153 regels, coverage 73% → 82%)
- coffeeshop → Uitgaan (was Dagelijks Overig)
- donkeyr → OV & Reizen (was Dagelijks Overig)
- Nieuw: hostel, booking.com, finnair, ns internationaal, apartt, tallinna (OV & Reizen)
- Nieuw: snackbar, horeca, rimi, zabka, narvesen, latvijas, restoran, comptoirs (Eten/Boodschappen)
- Nieuw: amare, escaperoom, museumkaart, hobby point, ballonnetje (Cultuur)
- Nieuw: smartshop, naughty squirrel, club storage (Uitgaan)
- Nieuw: klipper (Kapper), textielhuis, c&a (Kleding), infomedics (Gezondheid)
- Nieuw: boom uitgevers (Studie), kvk (Zakelijke Kosten), studentenuitzend (Salaris)
- Nieuw: renteafsluiting (Bankkosten), geldmaa / gea betaalpas (Dagelijks Overig)
- fix: geldmaat keyword → geldmaa (merchant wordt afgekapt in TAB export)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bookkeeping/rules.xlsx
+++ b/bookkeeping/rules.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B107"/>
+  <dimension ref="A1:B154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Dagelijks Overig</t>
+          <t>Uitgaan</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1085,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Dagelijks Overig</t>
+          <t>OV &amp; Reizen</t>
         </is>
       </c>
     </row>
@@ -1722,6 +1722,570 @@
       <c r="B107" t="inlineStr">
         <is>
           <t>Beleggen</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>hostel</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>booking.com</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>apartt</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>osada</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>snackbar</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>snackzone</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>horeca</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>narvesen</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>roi des belges</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>paviljoen</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>witte de with</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>latvijas</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>tabak and more</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>antik bufe</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>rimi</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Boodschappen</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>zabka</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Boodschappen</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>smartshop</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Uitgaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>naughty squirrel</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Uitgaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>hobby point</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Cultuur &amp; Entertainment</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>amare</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Cultuur &amp; Entertainment</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>sportsnutrition</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Gezondheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>bgs nutrition</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Gezondheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>bolcom</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Dagelijks Overig</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>geldmaa</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Dagelijks Overig</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>renteafsluiting</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Bankkosten</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>studentenuitzend</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Salaris</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>tallinna</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>turizm</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>bussijaam</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>k-market</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Boodschappen</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>maxima viru</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Boodschappen</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>restoran</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>sur restoran</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>klipper</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Kapper</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>club storage</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Uitgaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>ballonnetje</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Cultuur &amp; Entertainment</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>finnair</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>ns internationaal</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>OV &amp; Reizen</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>infomedics</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Gezondheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>escaperoom</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Cultuur &amp; Entertainment</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>museumkaart</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Cultuur &amp; Entertainment</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>textielhuis</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Kleding</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c&amp;a </t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Kleding</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>boom uitgevers</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Studie</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>comptoirs</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Eten &amp; Drinken</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>kvk</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Zakelijke Kosten</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>gea, betaalpas</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Dagelijks Overig</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: regels bijgewerkt o.b.v. handmatige categorisatie
- revolut → Interne Overboeking (eigen Revolut rekening, was Dagelijks Overig)
- revonl22 (BIC) als iban_rule → Interne Overboeking (SEPA naar Revolut IBAN)
- 12go → Sport & Fitness (12GO Biking)
- rlvnt → Sport & Fitness (Rlvnt Distribution sportswear)
- mediamarktsaturn → Zakelijke Kosten (PayPal/platform aankopen voor ODS)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bookkeeping/rules.xlsx
+++ b/bookkeeping/rules.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B154"/>
+  <dimension ref="A1:B157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Dagelijks Overig</t>
+          <t>Interne Overboeking</t>
         </is>
       </c>
     </row>
@@ -2286,6 +2286,42 @@
       <c r="B154" t="inlineStr">
         <is>
           <t>Dagelijks Overig</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>12go</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Sport &amp; Fitness</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>rlvnt</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Sport &amp; Fitness</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>mediamarktsaturn</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Zakelijke Kosten</t>
         </is>
       </c>
     </row>

</xml_diff>